<commit_message>
Refactor bridge API routes and update database schema and export templates
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/exports/Template_Fonte_Dados_Bridge_EBITDA.xlsx
+++ b/exports/Template_Fonte_Dados_Bridge_EBITDA.xlsx
@@ -5,9 +5,11 @@
   <sheets>
     <sheet name="Instruções" sheetId="1" r:id="rId1"/>
     <sheet name="Cenarios" sheetId="2" r:id="rId2"/>
-    <sheet name="Fatos" sheetId="3" r:id="rId3"/>
-    <sheet name="Detalhes" sheetId="4" r:id="rId4"/>
-    <sheet name="Metricas" sheetId="5" r:id="rId5"/>
+    <sheet name="Parametros" sheetId="3" r:id="rId3"/>
+    <sheet name="Vendas" sheetId="4" r:id="rId4"/>
+    <sheet name="CustoFixo" sheetId="5" r:id="rId5"/>
+    <sheet name="Insumos" sheetId="6" r:id="rId6"/>
+    <sheet name="Misc" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -401,86 +403,111 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A23"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>MODELO DA FONTE DE DADOS — PAINEL BRIDGE DE EBITDA</v>
+        <v>MODELO DA FONTE DE DADOS (DADOS BRUTOS) — PAINEL BRIDGE DE EBITDA</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Preencha as abas Cenarios, Fatos e Detalhes (esta última é opcional, usada no drill-down).</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>REGRAS DO MODELO:</v>
+        <v>O painel calcula todos os efeitos do bridge na hora da comparação, seguindo as fórmulas da aba 'Cálculo'.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>A fonte de dados só precisa trazer os dados brutos abaixo, por cenário (versão × período).</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>1. Cada cenário é uma combinação de VERSÃO (BUDGET, MRF1..MRF7) e PERÍODO (FY26, Q126..Q426, JAN26..DEC26).</v>
+        <v>REGRAS DO MODELO:</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2. tipo_periodo deve ser: year (ano), quarter (trimestre) ou month (mês). Só se comparam períodos do mesmo tipo.</v>
+        <v>1. Cada cenário é uma combinação de VERSÃO (BUDGET, MRF1..MRF7) e PERÍODO (FY26, Q126..Q426, JAN26..DEC26).</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>3. Na aba Fatos, cada cenário tem uma linha com metrica = ebitda (valor do EBITDA em MUSD)</v>
+        <v>2. tipo_periodo deve ser: year (ano), quarter (trimestre) ou month (mês). Só se comparam períodos do mesmo tipo.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v xml:space="preserve">   e uma linha por alavanca com o NÍVEL ACUMULADO relativo à referência (BUDGET = 0).</v>
+        <v>3. Aba Parametros — uma linha por cenário:</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v xml:space="preserve">   Ex.: se o preço de venda do MRF7 está 286,5 MUSD acima do Budget, a linha selling_price do MRF7 vale 286,5.</v>
+        <v xml:space="preserve">   cambio: BRL/USD médio do período | cambio_custo_fixo: câmbio usado no bloco de custo fixo (pode diferir levemente)</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>4. Consistência obrigatória: ebitda do cenário = ebitda da referência + soma dos níveis das alavancas.</v>
+        <v xml:space="preserve">   aco_bruto_kt: produção de aço bruto (kt) | ebitda_kusd: EBITDA do cenário em kUSD | participacao_custo_dm: fração do custo em moeda local (padrão 0,4).</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v xml:space="preserve">   Assim, o bridge de qualquer par origem→destino fecha exatamente (destino − origem por alavanca).</v>
+        <v>4. Aba Vendas — uma linha por produto por cenário:</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>5. Alavancas com nível zero podem ser omitidas.</v>
+        <v xml:space="preserve">   qtd_t: quantidade (t) | faturamento_kusd: receita (kUSD) | custo_variavel_kusd: custo variável (kUSD)</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>6. Na aba Detalhes, as linhas de cada alavanca de um cenário devem somar o nível daquela alavanca.</v>
+        <v xml:space="preserve">   moeda: BRL (preço formado em real) ou USD | mercado_interno: TRUE para vendas domésticas (expostas a câmbio).</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v xml:space="preserve">   Linhas ausentes em um dos cenários são tratadas como zero na comparação.</v>
+        <v xml:space="preserve">   Produtos novos (qtd zero na referência) são tratados automaticamente: efeito só em volume/mix e câmbio.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>7. Valores sempre em MUSD (milhões de dólares).</v>
+        <v>5. Aba CustoFixo — montante (kUSD) por categoria; usd: TRUE quando a categoria é denominada em USD (sem efeito câmbio).</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>6. Aba Insumos — itens com preço: preco_usd (USD/unidade) e rendimento (consumo por t de aço); o efeito usa a produção de aço bruto.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
+        <v xml:space="preserve">   Itens sem preço: informar montante_kusd direto (o efeito é a diferença entre cenários).</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>7. Aba Misc — alavanca = usage (consumo), others (outros, ex.: Logística/VAT) ou stock_variation (itens de variação de estoque).</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v xml:space="preserve">   A variação de estoque recebe também o ajuste de fechamento: o bridge sempre fecha exatamente no EBITDA informado.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>8. Unidades: montantes em kUSD (milhares de USD); o painel apresenta em MUSD.</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
         <v>As abas contêm exemplos reais de FY26 Budget (referência) e FY26 MRF7 (632,0 → 747,7 MUSD).</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A23"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3238,727 +3265,947 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:F3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>cenario_id</v>
       </c>
       <c r="B1" t="str">
-        <v>metrica</v>
+        <v>cambio</v>
       </c>
       <c r="C1" t="str">
-        <v>valor_musd</v>
+        <v>cambio_custo_fixo</v>
+      </c>
+      <c r="D1" t="str">
+        <v>aco_bruto_kt</v>
+      </c>
+      <c r="E1" t="str">
+        <v>ebitda_kusd</v>
+      </c>
+      <c r="F1" t="str">
+        <v>participacao_custo_dm</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
         <v>fy26_fy_budget</v>
       </c>
-      <c r="B2" t="str">
-        <v>ebitda</v>
+      <c r="B2">
+        <v>5.3999999999999995</v>
       </c>
       <c r="C2">
-        <v>632.0440445298751</v>
+        <v>5.3999999999999995</v>
+      </c>
+      <c r="D2">
+        <v>6970285.66</v>
+      </c>
+      <c r="E2">
+        <v>632044.044529875</v>
+      </c>
+      <c r="F2">
+        <v>0.4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
         <v>fy26_fy_mrf7</v>
       </c>
-      <c r="B3" t="str">
-        <v>ebitda</v>
+      <c r="B3">
+        <v>5.17621443903319</v>
       </c>
       <c r="C3">
-        <v>747.6924008767779</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>fy26_fy_mrf7</v>
-      </c>
-      <c r="B4" t="str">
-        <v>vol_mix</v>
-      </c>
-      <c r="C4">
-        <v>-6.680380721635153</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>fy26_fy_mrf7</v>
-      </c>
-      <c r="B5" t="str">
-        <v>selling_price</v>
-      </c>
-      <c r="C5">
-        <v>286.5489436934462</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>fy26_fy_mrf7</v>
-      </c>
-      <c r="B6" t="str">
-        <v>input_price</v>
-      </c>
-      <c r="C6">
-        <v>-177.47194678166522</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>fy26_fy_mrf7</v>
-      </c>
-      <c r="B7" t="str">
-        <v>usage</v>
-      </c>
-      <c r="C7">
-        <v>-12.829343372386798</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>fy26_fy_mrf7</v>
-      </c>
-      <c r="B8" t="str">
-        <v>fixed_cost</v>
-      </c>
-      <c r="C8">
-        <v>-34.29055851516902</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>fy26_fy_mrf7</v>
-      </c>
-      <c r="B9" t="str">
-        <v>forex</v>
-      </c>
-      <c r="C9">
-        <v>70.572858606569</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>fy26_fy_mrf7</v>
-      </c>
-      <c r="B10" t="str">
-        <v>sv_others</v>
-      </c>
-      <c r="C10">
-        <v>-10.201216562256178</v>
+        <v>5.173745409366377</v>
+      </c>
+      <c r="D3">
+        <v>6970285.66</v>
+      </c>
+      <c r="E3">
+        <v>747692.400876778</v>
+      </c>
+      <c r="F3">
+        <v>0.4</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:I59"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>cenario_id</v>
       </c>
       <c r="B1" t="str">
-        <v>alavanca</v>
+        <v>produto</v>
       </c>
       <c r="C1" t="str">
-        <v>linha</v>
+        <v>rotulo</v>
       </c>
       <c r="D1" t="str">
-        <v>grupo</v>
+        <v>moeda</v>
       </c>
       <c r="E1" t="str">
-        <v>valor_musd</v>
+        <v>mercado_interno</v>
       </c>
       <c r="F1" t="str">
+        <v>qtd_t</v>
+      </c>
+      <c r="G1" t="str">
+        <v>faturamento_kusd</v>
+      </c>
+      <c r="H1" t="str">
+        <v>custo_variavel_kusd</v>
+      </c>
+      <c r="I1" t="str">
         <v>ordem</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B2" t="str">
-        <v>vol_mix</v>
+        <v>slab_calvert</v>
       </c>
       <c r="C2" t="str">
-        <v>Volume</v>
+        <v>Slab Calvert</v>
       </c>
       <c r="D2" t="str">
-        <v>Resumo</v>
-      </c>
-      <c r="E2">
-        <v>-23.126221100435135</v>
+        <v>USD</v>
+      </c>
+      <c r="E2" t="b">
+        <v>0</v>
       </c>
       <c r="F2">
+        <v>961000</v>
+      </c>
+      <c r="G2">
+        <v>501302.49550381646</v>
+      </c>
+      <c r="H2">
+        <v>420316.4611155691</v>
+      </c>
+      <c r="I2">
         <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B3" t="str">
-        <v>selling_price</v>
+        <v>slabs_others_intragroup</v>
       </c>
       <c r="C3" t="str">
-        <v>Slab Calvert</v>
+        <v>Slabs Others Intragroup</v>
       </c>
       <c r="D3" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E3">
-        <v>87.29303862594274</v>
+        <v>USD</v>
+      </c>
+      <c r="E3" t="b">
+        <v>0</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>400000</v>
+      </c>
+      <c r="G3">
+        <v>177829.60148671025</v>
+      </c>
+      <c r="H3">
+        <v>166549.61961105894</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B4" t="str">
-        <v>forex</v>
+        <v>slabs_3rd_party</v>
       </c>
       <c r="C4" t="str">
-        <v>HRC DM Industry</v>
+        <v>Slabs 3rd Party</v>
       </c>
       <c r="D4" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E4">
-        <v>41.457031146283676</v>
+        <v>USD</v>
+      </c>
+      <c r="E4" t="b">
+        <v>0</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>1423164.3800000001</v>
+      </c>
+      <c r="G4">
+        <v>645093.3753540799</v>
+      </c>
+      <c r="H4">
+        <v>592568.7153325214</v>
+      </c>
+      <c r="I4">
+        <v>2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B5" t="str">
-        <v>sv_others</v>
+        <v>slab_dm</v>
       </c>
       <c r="C5" t="str">
-        <v>Outros (Others)</v>
+        <v>Slab DM</v>
       </c>
       <c r="D5" t="str">
-        <v/>
-      </c>
-      <c r="E5">
-        <v>-5.7640203629386235</v>
+        <v>BRL</v>
+      </c>
+      <c r="E5" t="b">
+        <v>1</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>31000.000000000004</v>
+      </c>
+      <c r="G5">
+        <v>13984.147709531153</v>
+      </c>
+      <c r="H5">
+        <v>13961.595519857068</v>
+      </c>
+      <c r="I5">
+        <v>3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B6" t="str">
-        <v>input_price</v>
+        <v>plates_dm</v>
       </c>
       <c r="C6" t="str">
-        <v>Total preço de insumos (aba Cálculo)</v>
+        <v>Plates DM</v>
       </c>
       <c r="D6" t="str">
-        <v/>
-      </c>
-      <c r="E6">
-        <v>-177.47194678166522</v>
+        <v>BRL</v>
+      </c>
+      <c r="E6" t="b">
+        <v>1</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>18000</v>
+      </c>
+      <c r="G6">
+        <v>12337.203108910493</v>
+      </c>
+      <c r="H6">
+        <v>7494.732882497652</v>
+      </c>
+      <c r="I6">
+        <v>4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B7" t="str">
-        <v>usage</v>
+        <v>hrc_export</v>
       </c>
       <c r="C7" t="str">
-        <v>Total consumo (aba Cálculo)</v>
+        <v>HRC Export</v>
       </c>
       <c r="D7" t="str">
-        <v/>
-      </c>
-      <c r="E7">
-        <v>-12.829343372386798</v>
+        <v>USD</v>
+      </c>
+      <c r="E7" t="b">
+        <v>0</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>433467</v>
+      </c>
+      <c r="G7">
+        <v>209045.75207432156</v>
+      </c>
+      <c r="H7">
+        <v>193418.28573904067</v>
+      </c>
+      <c r="I7">
+        <v>5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B8" t="str">
-        <v>fixed_cost</v>
+        <v>hrc_dm_auto</v>
       </c>
       <c r="C8" t="str">
-        <v>Total custo fixo (aba Cálculo)</v>
+        <v>HRC DM Auto</v>
       </c>
       <c r="D8" t="str">
-        <v/>
-      </c>
-      <c r="E8">
-        <v>-34.29055851516902</v>
+        <v>BRL</v>
+      </c>
+      <c r="E8" t="b">
+        <v>1</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>85817.96</v>
+      </c>
+      <c r="G8">
+        <v>58479.86744174038</v>
+      </c>
+      <c r="H8">
+        <v>37520.66345492433</v>
+      </c>
+      <c r="I8">
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B9" t="str">
-        <v>vol_mix</v>
+        <v>hrc_dm_industry</v>
       </c>
       <c r="C9" t="str">
-        <v>Mix</v>
+        <v>HRC DM Industry</v>
       </c>
       <c r="D9" t="str">
-        <v>Resumo</v>
-      </c>
-      <c r="E9">
-        <v>16.445840378799982</v>
+        <v>BRL</v>
+      </c>
+      <c r="E9" t="b">
+        <v>1</v>
       </c>
       <c r="F9">
-        <v>1</v>
+        <v>1438681.32</v>
+      </c>
+      <c r="G9">
+        <v>947762.9877364037</v>
+      </c>
+      <c r="H9">
+        <v>629009.0981725305</v>
+      </c>
+      <c r="I9">
+        <v>7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B10" t="str">
-        <v>selling_price</v>
+        <v>hrc_dm_downstream</v>
       </c>
       <c r="C10" t="str">
-        <v>Slabs Others Intragroup</v>
+        <v>HRC DM Downstream</v>
       </c>
       <c r="D10" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E10">
-        <v>71.85081374420872</v>
+        <v>BRL</v>
+      </c>
+      <c r="E10" t="b">
+        <v>1</v>
       </c>
       <c r="F10">
-        <v>1</v>
+        <v>427373.81000000006</v>
+      </c>
+      <c r="G10">
+        <v>322882.6888881808</v>
+      </c>
+      <c r="H10">
+        <v>221042.9702242862</v>
+      </c>
+      <c r="I10">
+        <v>8</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B11" t="str">
-        <v>forex</v>
+        <v>p_o_dm_auto</v>
       </c>
       <c r="C11" t="str">
-        <v>HDG DM Auto</v>
+        <v>P&amp;O DM Auto</v>
       </c>
       <c r="D11" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E11">
-        <v>21.120061170754283</v>
+        <v>BRL</v>
+      </c>
+      <c r="E11" t="b">
+        <v>1</v>
       </c>
       <c r="F11">
-        <v>1</v>
+        <v>102999.19000000002</v>
+      </c>
+      <c r="G11">
+        <v>88497.53332715324</v>
+      </c>
+      <c r="H11">
+        <v>53272.44289558969</v>
+      </c>
+      <c r="I11">
+        <v>9</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B12" t="str">
-        <v>sv_others</v>
+        <v>p_o_dm_industry</v>
       </c>
       <c r="C12" t="str">
-        <v>Variação de estoque</v>
+        <v>P&amp;O DM Industry</v>
       </c>
       <c r="D12" t="str">
-        <v/>
-      </c>
-      <c r="E12">
-        <v>-4.437196199317555</v>
+        <v>BRL</v>
+      </c>
+      <c r="E12" t="b">
+        <v>1</v>
       </c>
       <c r="F12">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>10</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B13" t="str">
-        <v>vol_mix</v>
+        <v>crc_em_auto</v>
       </c>
       <c r="C13" t="str">
-        <v>Slabs 3rd Party</v>
+        <v>CRC EM Auto</v>
       </c>
       <c r="D13" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E13">
-        <v>-20.253772902400698</v>
+        <v>BRL</v>
+      </c>
+      <c r="E13" t="b">
+        <v>1</v>
       </c>
       <c r="F13">
-        <v>2</v>
+        <v>1220.3923579624538</v>
+      </c>
+      <c r="G13">
+        <v>1077.5971012541204</v>
+      </c>
+      <c r="H13">
+        <v>603.7574182612613</v>
+      </c>
+      <c r="I13">
+        <v>11</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B14" t="str">
-        <v>selling_price</v>
+        <v>crc_em_industry</v>
       </c>
       <c r="C14" t="str">
-        <v>Slabs 3rd Party</v>
+        <v>CRC EM Industry</v>
       </c>
       <c r="D14" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E14">
-        <v>58.62051354862707</v>
+        <v>USD</v>
+      </c>
+      <c r="E14" t="b">
+        <v>0</v>
       </c>
       <c r="F14">
-        <v>2</v>
+        <v>492.26</v>
+      </c>
+      <c r="G14">
+        <v>159.1550089907945</v>
+      </c>
+      <c r="H14">
+        <v>243.53284808297053</v>
+      </c>
+      <c r="I14">
+        <v>12</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B15" t="str">
-        <v>forex</v>
+        <v>crc_dm_auto</v>
       </c>
       <c r="C15" t="str">
-        <v>HDG DM Industry</v>
+        <v>CRC DM Auto</v>
       </c>
       <c r="D15" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E15">
-        <v>16.587596535791338</v>
+        <v>BRL</v>
+      </c>
+      <c r="E15" t="b">
+        <v>1</v>
       </c>
       <c r="F15">
-        <v>2</v>
+        <v>90127.47039519616</v>
+      </c>
+      <c r="G15">
+        <v>83099.53095645981</v>
+      </c>
+      <c r="H15">
+        <v>44588.224832112566</v>
+      </c>
+      <c r="I15">
+        <v>13</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B16" t="str">
-        <v>vol_mix</v>
+        <v>crc_dm_industry</v>
       </c>
       <c r="C16" t="str">
-        <v>Slabs Others Intragroup</v>
+        <v>CRC DM Industry</v>
       </c>
       <c r="D16" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E16">
-        <v>16.844596653046928</v>
+        <v>BRL</v>
+      </c>
+      <c r="E16" t="b">
+        <v>1</v>
       </c>
       <c r="F16">
-        <v>3</v>
+        <v>265325.5399999999</v>
+      </c>
+      <c r="G16">
+        <v>209133.77960682815</v>
+      </c>
+      <c r="H16">
+        <v>131262.91883425854</v>
+      </c>
+      <c r="I16">
+        <v>14</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B17" t="str">
-        <v>selling_price</v>
+        <v>crc_dm_downstream</v>
       </c>
       <c r="C17" t="str">
-        <v>HRC DM Industry</v>
+        <v>CRC DM Downstream</v>
       </c>
       <c r="D17" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E17">
-        <v>50.57003338274117</v>
+        <v>BRL</v>
+      </c>
+      <c r="E17" t="b">
+        <v>1</v>
       </c>
       <c r="F17">
-        <v>3</v>
+        <v>110301.97000000002</v>
+      </c>
+      <c r="G17">
+        <v>91936.73824458114</v>
+      </c>
+      <c r="H17">
+        <v>63393.192059965026</v>
+      </c>
+      <c r="I17">
+        <v>15</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B18" t="str">
-        <v>forex</v>
+        <v>hdg_em_auto</v>
       </c>
       <c r="C18" t="str">
-        <v>HRC DM Downstream</v>
+        <v>HDG EM Auto</v>
       </c>
       <c r="D18" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E18">
-        <v>14.79596241334703</v>
+        <v>BRL</v>
+      </c>
+      <c r="E18" t="b">
+        <v>1</v>
       </c>
       <c r="F18">
-        <v>3</v>
+        <v>49551.85324452803</v>
+      </c>
+      <c r="G18">
+        <v>50444.68127719643</v>
+      </c>
+      <c r="H18">
+        <v>28371.53293992054</v>
+      </c>
+      <c r="I18">
+        <v>16</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B19" t="str">
-        <v>vol_mix</v>
+        <v>hdg_em_industry</v>
       </c>
       <c r="C19" t="str">
-        <v>AlZn DM Industry</v>
+        <v>HDG EM Industry</v>
       </c>
       <c r="D19" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E19">
-        <v>-13.9695915562111</v>
+        <v>USD</v>
+      </c>
+      <c r="E19" t="b">
+        <v>0</v>
       </c>
       <c r="F19">
-        <v>4</v>
+        <v>1014.1200000000001</v>
+      </c>
+      <c r="G19">
+        <v>327.8801400027313</v>
+      </c>
+      <c r="H19">
+        <v>600.5665879113399</v>
+      </c>
+      <c r="I19">
+        <v>17</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B20" t="str">
-        <v>selling_price</v>
+        <v>hdg_dm_auto</v>
       </c>
       <c r="C20" t="str">
-        <v>HDG DM Industry</v>
+        <v>HDG DM Auto</v>
       </c>
       <c r="D20" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E20">
-        <v>27.970262821155195</v>
+        <v>BRL</v>
+      </c>
+      <c r="E20" t="b">
+        <v>1</v>
       </c>
       <c r="F20">
-        <v>4</v>
+        <v>463694.02845894557</v>
+      </c>
+      <c r="G20">
+        <v>484605.9861422443</v>
+      </c>
+      <c r="H20">
+        <v>265493.8118569804</v>
+      </c>
+      <c r="I20">
+        <v>18</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B21" t="str">
-        <v>forex</v>
+        <v>hdg_dm_industry</v>
       </c>
       <c r="C21" t="str">
-        <v>CRC DM Industry</v>
+        <v>HDG DM Industry</v>
       </c>
       <c r="D21" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E21">
-        <v>10.018396072049008</v>
+        <v>BRL</v>
+      </c>
+      <c r="E21" t="b">
+        <v>1</v>
       </c>
       <c r="F21">
-        <v>4</v>
+        <v>416584.70999999996</v>
+      </c>
+      <c r="G21">
+        <v>353590.0008385644</v>
+      </c>
+      <c r="H21">
+        <v>246703.40577124502</v>
+      </c>
+      <c r="I21">
+        <v>19</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B22" t="str">
-        <v>vol_mix</v>
+        <v>hdg_dm_downstream</v>
       </c>
       <c r="C22" t="str">
-        <v>P&amp;O DM Industry</v>
+        <v>HDG DM Downstream</v>
       </c>
       <c r="D22" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E22">
-        <v>12.236762966391787</v>
+        <v>BRL</v>
+      </c>
+      <c r="E22" t="b">
+        <v>1</v>
       </c>
       <c r="F22">
-        <v>5</v>
+        <v>83539.32999999999</v>
+      </c>
+      <c r="G22">
+        <v>73539.84552044267</v>
+      </c>
+      <c r="H22">
+        <v>56155.52676376309</v>
+      </c>
+      <c r="I22">
+        <v>20</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B23" t="str">
-        <v>selling_price</v>
+        <v>alzn_dm_industry</v>
       </c>
       <c r="C23" t="str">
-        <v>HDG DM Auto</v>
+        <v>AlZn DM Industry</v>
       </c>
       <c r="D23" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E23">
-        <v>24.928758284361457</v>
+        <v>BRL</v>
+      </c>
+      <c r="E23" t="b">
+        <v>1</v>
       </c>
       <c r="F23">
-        <v>5</v>
+        <v>181457.09000000003</v>
+      </c>
+      <c r="G23">
+        <v>176561.66966426402</v>
+      </c>
+      <c r="H23">
+        <v>120461.97847755178</v>
+      </c>
+      <c r="I23">
+        <v>22</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B24" t="str">
-        <v>forex</v>
+        <v>alzn_dm_downstream</v>
       </c>
       <c r="C24" t="str">
-        <v>AlZn DM Industry</v>
+        <v>ALZn DM Downstream</v>
       </c>
       <c r="D24" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E24">
-        <v>5.8034423521044545</v>
+        <v>BRL</v>
+      </c>
+      <c r="E24" t="b">
+        <v>1</v>
       </c>
       <c r="F24">
-        <v>5</v>
+        <v>106335.88</v>
+      </c>
+      <c r="G24">
+        <v>115705.20290064352</v>
+      </c>
+      <c r="H24">
+        <v>79098.93427555055</v>
+      </c>
+      <c r="I24">
+        <v>23</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B25" t="str">
-        <v>vol_mix</v>
+        <v>usibor_dm_auto</v>
       </c>
       <c r="C25" t="str">
-        <v>HRC Export</v>
+        <v>Usibor DM Auto</v>
       </c>
       <c r="D25" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E25">
-        <v>-8.504735358024249</v>
+        <v>BRL</v>
+      </c>
+      <c r="E25" t="b">
+        <v>1</v>
       </c>
       <c r="F25">
-        <v>6</v>
+        <v>94231.59468414272</v>
+      </c>
+      <c r="G25">
+        <v>121687.95556710853</v>
+      </c>
+      <c r="H25">
+        <v>53979.88030619434</v>
+      </c>
+      <c r="I25">
+        <v>24</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B26" t="str">
-        <v>selling_price</v>
+        <v>alsi_dm_industry</v>
       </c>
       <c r="C26" t="str">
-        <v>HRC DM Downstream</v>
+        <v>AlSi DM Industry</v>
       </c>
       <c r="D26" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E26">
-        <v>19.803763687314547</v>
+        <v>BRL</v>
+      </c>
+      <c r="E26" t="b">
+        <v>1</v>
       </c>
       <c r="F26">
-        <v>6</v>
+        <v>7737.539999999999</v>
+      </c>
+      <c r="G26">
+        <v>6566.996903879877</v>
+      </c>
+      <c r="H26">
+        <v>4432.393237792426</v>
+      </c>
+      <c r="I26">
+        <v>25</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B27" t="str">
-        <v>forex</v>
+        <v>auto_imports_pp_dm</v>
       </c>
       <c r="C27" t="str">
-        <v>Usibor DM Auto</v>
+        <v>Auto Imports/PP DM</v>
       </c>
       <c r="D27" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E27">
-        <v>5.685398755362816</v>
+        <v>BRL</v>
+      </c>
+      <c r="E27" t="b">
+        <v>1</v>
       </c>
       <c r="F27">
-        <v>6</v>
+        <v>3816.3261818387646</v>
+      </c>
+      <c r="G27">
+        <v>7146.0046210960845</v>
+      </c>
+      <c r="H27">
+        <v>2533.503664034172</v>
+      </c>
+      <c r="I27">
+        <v>26</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B28" t="str">
-        <v>vol_mix</v>
+        <v>magnelis_dm_industry</v>
       </c>
       <c r="C28" t="str">
-        <v>ALZn DM Downstream</v>
+        <v>Magnelis DM Industry</v>
       </c>
       <c r="D28" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E28">
-        <v>-6.131981376050678</v>
+        <v>USD</v>
+      </c>
+      <c r="E28" t="b">
+        <v>0</v>
       </c>
       <c r="F28">
-        <v>7</v>
+        <v>0</v>
+      </c>
+      <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28">
+        <v>0</v>
+      </c>
+      <c r="I28">
+        <v>27</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B29" t="str">
-        <v>selling_price</v>
+        <v>industry_imports</v>
       </c>
       <c r="C29" t="str">
-        <v>CRC DM Industry</v>
+        <v>Industry Imports</v>
       </c>
       <c r="D29" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E29">
-        <v>16.22020453157885</v>
+        <v>BRL</v>
+      </c>
+      <c r="E29" t="b">
+        <v>1</v>
       </c>
       <c r="F29">
-        <v>7</v>
+        <v>35399.96999999999</v>
+      </c>
+      <c r="G29">
+        <v>33584.623171525105</v>
+      </c>
+      <c r="H29">
+        <v>23500.599641744375</v>
+      </c>
+      <c r="I29">
+        <v>28</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>fy26_fy_mrf7</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B30" t="str">
-        <v>forex</v>
+        <v>magnelis_dm_downstream</v>
       </c>
       <c r="C30" t="str">
-        <v>ALZn DM Downstream</v>
+        <v>Magnelis DM Downstream</v>
       </c>
       <c r="D30" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E30">
-        <v>4.344987126740586</v>
+        <v>BRL</v>
+      </c>
+      <c r="E30" t="b">
+        <v>1</v>
       </c>
       <c r="F30">
-        <v>7</v>
+        <v>0</v>
+      </c>
+      <c r="G30">
+        <v>0</v>
+      </c>
+      <c r="H30">
+        <v>0</v>
+      </c>
+      <c r="I30">
+        <v>29</v>
       </c>
     </row>
     <row r="31">
@@ -3966,19 +4213,28 @@
         <v>fy26_fy_mrf7</v>
       </c>
       <c r="B31" t="str">
-        <v>vol_mix</v>
+        <v>slab_calvert</v>
       </c>
       <c r="C31" t="str">
-        <v>CRC DM Industry</v>
+        <v>Slab Calvert</v>
       </c>
       <c r="D31" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E31">
-        <v>6.103683176804887</v>
+        <v>USD</v>
+      </c>
+      <c r="E31" t="b">
+        <v>0</v>
       </c>
       <c r="F31">
-        <v>8</v>
+        <v>966247.8699999999</v>
+      </c>
+      <c r="G31">
+        <v>591333.0682890512</v>
+      </c>
+      <c r="H31">
+        <v>422611.74326623976</v>
+      </c>
+      <c r="I31">
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -3986,19 +4242,28 @@
         <v>fy26_fy_mrf7</v>
       </c>
       <c r="B32" t="str">
-        <v>selling_price</v>
+        <v>slabs_others_intragroup</v>
       </c>
       <c r="C32" t="str">
-        <v>HRC Export</v>
+        <v>Slabs Others Intragroup</v>
       </c>
       <c r="D32" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E32">
-        <v>14.779689222688518</v>
+        <v>USD</v>
+      </c>
+      <c r="E32" t="b">
+        <v>0</v>
       </c>
       <c r="F32">
-        <v>8</v>
+        <v>997327.082214813</v>
+      </c>
+      <c r="G32">
+        <v>515236.507699618</v>
+      </c>
+      <c r="H32">
+        <v>415261.11542671104</v>
+      </c>
+      <c r="I32">
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -4006,19 +4271,28 @@
         <v>fy26_fy_mrf7</v>
       </c>
       <c r="B33" t="str">
-        <v>forex</v>
+        <v>slabs_3rd_party</v>
       </c>
       <c r="C33" t="str">
-        <v>CRC DM Downstream</v>
+        <v>Slabs 3rd Party</v>
       </c>
       <c r="D33" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E33">
-        <v>4.340361852603534</v>
+        <v>USD</v>
+      </c>
+      <c r="E33" t="b">
+        <v>0</v>
       </c>
       <c r="F33">
-        <v>8</v>
+        <v>874385.0420000006</v>
+      </c>
+      <c r="G33">
+        <v>454962.6410145345</v>
+      </c>
+      <c r="H33">
+        <v>364071.2403467497</v>
+      </c>
+      <c r="I33">
+        <v>2</v>
       </c>
     </row>
     <row r="34">
@@ -4026,19 +4300,28 @@
         <v>fy26_fy_mrf7</v>
       </c>
       <c r="B34" t="str">
-        <v>vol_mix</v>
+        <v>slab_dm</v>
       </c>
       <c r="C34" t="str">
-        <v>HDG DM Industry</v>
+        <v>Slab DM</v>
       </c>
       <c r="D34" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E34">
-        <v>5.653564201977188</v>
+        <v>BRL</v>
+      </c>
+      <c r="E34" t="b">
+        <v>1</v>
       </c>
       <c r="F34">
-        <v>9</v>
+        <v>32424.16</v>
+      </c>
+      <c r="G34">
+        <v>15058.548634938072</v>
+      </c>
+      <c r="H34">
+        <v>14603.000225520282</v>
+      </c>
+      <c r="I34">
+        <v>3</v>
       </c>
     </row>
     <row r="35">
@@ -4046,19 +4329,28 @@
         <v>fy26_fy_mrf7</v>
       </c>
       <c r="B35" t="str">
-        <v>selling_price</v>
+        <v>plates_dm</v>
       </c>
       <c r="C35" t="str">
-        <v>Usibor DM Auto</v>
+        <v>Plates DM</v>
       </c>
       <c r="D35" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E35">
-        <v>8.927178406925167</v>
+        <v>BRL</v>
+      </c>
+      <c r="E35" t="b">
+        <v>1</v>
       </c>
       <c r="F35">
-        <v>9</v>
+        <v>16529.159999999996</v>
+      </c>
+      <c r="G35">
+        <v>11582.35072808389</v>
+      </c>
+      <c r="H35">
+        <v>6882.313276225826</v>
+      </c>
+      <c r="I35">
+        <v>4</v>
       </c>
     </row>
     <row r="36">
@@ -4066,19 +4358,28 @@
         <v>fy26_fy_mrf7</v>
       </c>
       <c r="B36" t="str">
-        <v>forex</v>
+        <v>hrc_export</v>
       </c>
       <c r="C36" t="str">
-        <v>CRC DM Auto</v>
+        <v>HRC Export</v>
       </c>
       <c r="D36" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E36">
-        <v>3.8953735808122136</v>
+        <v>USD</v>
+      </c>
+      <c r="E36" t="b">
+        <v>0</v>
       </c>
       <c r="F36">
-        <v>9</v>
+        <v>197566.82000000007</v>
+      </c>
+      <c r="G36">
+        <v>110059.15564535075</v>
+      </c>
+      <c r="H36">
+        <v>88156.73544540559</v>
+      </c>
+      <c r="I36">
+        <v>5</v>
       </c>
     </row>
     <row r="37">
@@ -4086,19 +4387,28 @@
         <v>fy26_fy_mrf7</v>
       </c>
       <c r="B37" t="str">
-        <v>vol_mix</v>
+        <v>hrc_dm_auto</v>
       </c>
       <c r="C37" t="str">
-        <v>Industry Imports</v>
+        <v>HRC DM Auto</v>
       </c>
       <c r="D37" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E37">
-        <v>-5.193191630739251</v>
+        <v>BRL</v>
+      </c>
+      <c r="E37" t="b">
+        <v>1</v>
       </c>
       <c r="F37">
-        <v>10</v>
+        <v>100236.84017419748</v>
+      </c>
+      <c r="G37">
+        <v>72754.90220446786</v>
+      </c>
+      <c r="H37">
+        <v>43824.77451061645</v>
+      </c>
+      <c r="I37">
+        <v>6</v>
       </c>
     </row>
     <row r="38">
@@ -4106,19 +4416,28 @@
         <v>fy26_fy_mrf7</v>
       </c>
       <c r="B38" t="str">
-        <v>selling_price</v>
+        <v>hrc_dm_industry</v>
       </c>
       <c r="C38" t="str">
-        <v>Demais itens e ajustes</v>
+        <v>HRC DM Industry</v>
       </c>
       <c r="D38" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E38">
-        <v>-94.41531256209731</v>
+        <v>BRL</v>
+      </c>
+      <c r="E38" t="b">
+        <v>1</v>
       </c>
       <c r="F38">
-        <v>10</v>
+        <v>1441770.7359999982</v>
+      </c>
+      <c r="G38">
+        <v>1000368.2419132253</v>
+      </c>
+      <c r="H38">
+        <v>630359.8286957005</v>
+      </c>
+      <c r="I38">
+        <v>7</v>
       </c>
     </row>
     <row r="39">
@@ -4126,19 +4445,28 @@
         <v>fy26_fy_mrf7</v>
       </c>
       <c r="B39" t="str">
-        <v>forex</v>
+        <v>hrc_dm_downstream</v>
       </c>
       <c r="C39" t="str">
-        <v>Demais itens e ajustes</v>
+        <v>HRC DM Downstream</v>
       </c>
       <c r="D39" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E39">
-        <v>-57.475752399279955</v>
+        <v>BRL</v>
+      </c>
+      <c r="E39" t="b">
+        <v>1</v>
       </c>
       <c r="F39">
-        <v>10</v>
+        <v>446359.43442400004</v>
+      </c>
+      <c r="G39">
+        <v>357030.1706995475</v>
+      </c>
+      <c r="H39">
+        <v>230862.56776640913</v>
+      </c>
+      <c r="I39">
+        <v>8</v>
       </c>
     </row>
     <row r="40">
@@ -4146,19 +4474,28 @@
         <v>fy26_fy_mrf7</v>
       </c>
       <c r="B40" t="str">
-        <v>vol_mix</v>
+        <v>p_o_dm_auto</v>
       </c>
       <c r="C40" t="str">
-        <v>HRC DM Downstream</v>
+        <v>P&amp;O DM Auto</v>
       </c>
       <c r="D40" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E40">
-        <v>4.524120581929258</v>
+        <v>BRL</v>
+      </c>
+      <c r="E40" t="b">
+        <v>1</v>
       </c>
       <c r="F40">
-        <v>11</v>
+        <v>90523.8577247</v>
+      </c>
+      <c r="G40">
+        <v>82781.52277303312</v>
+      </c>
+      <c r="H40">
+        <v>46820.048209384615</v>
+      </c>
+      <c r="I40">
+        <v>9</v>
       </c>
     </row>
     <row r="41">
@@ -4166,107 +4503,1826 @@
         <v>fy26_fy_mrf7</v>
       </c>
       <c r="B41" t="str">
-        <v>vol_mix</v>
+        <v>p_o_dm_industry</v>
       </c>
       <c r="C41" t="str">
-        <v>Demais itens e ajustes</v>
+        <v>P&amp;O DM Industry</v>
       </c>
       <c r="D41" t="str">
-        <v>Por produto</v>
-      </c>
-      <c r="E41">
-        <v>2.0101645216407746</v>
+        <v>BRL</v>
+      </c>
+      <c r="E41" t="b">
+        <v>1</v>
       </c>
       <c r="F41">
+        <v>45424.20800000002</v>
+      </c>
+      <c r="G41">
+        <v>32853.85332246733</v>
+      </c>
+      <c r="H41">
+        <v>20617.090356075543</v>
+      </c>
+      <c r="I41">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B42" t="str">
+        <v>crc_em_auto</v>
+      </c>
+      <c r="C42" t="str">
+        <v>CRC EM Auto</v>
+      </c>
+      <c r="D42" t="str">
+        <v>BRL</v>
+      </c>
+      <c r="E42" t="b">
+        <v>1</v>
+      </c>
+      <c r="F42">
+        <v>1887.810550681587</v>
+      </c>
+      <c r="G42">
+        <v>1769.2316837232268</v>
+      </c>
+      <c r="H42">
+        <v>933.945232293032</v>
+      </c>
+      <c r="I42">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B43" t="str">
+        <v>crc_em_industry</v>
+      </c>
+      <c r="C43" t="str">
+        <v>CRC EM Industry</v>
+      </c>
+      <c r="D43" t="str">
+        <v>USD</v>
+      </c>
+      <c r="E43" t="b">
+        <v>0</v>
+      </c>
+      <c r="F43">
+        <v>4847.375</v>
+      </c>
+      <c r="G43">
+        <v>2925.504307265212</v>
+      </c>
+      <c r="H43">
+        <v>2398.112866119915</v>
+      </c>
+      <c r="I43">
         <v>12</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B44" t="str">
+        <v>crc_dm_auto</v>
+      </c>
+      <c r="C44" t="str">
+        <v>CRC DM Auto</v>
+      </c>
+      <c r="D44" t="str">
+        <v>BRL</v>
+      </c>
+      <c r="E44" t="b">
+        <v>1</v>
+      </c>
+      <c r="F44">
+        <v>95622.29321562513</v>
+      </c>
+      <c r="G44">
+        <v>93996.31167225182</v>
+      </c>
+      <c r="H44">
+        <v>47306.645689322926</v>
+      </c>
+      <c r="I44">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B45" t="str">
+        <v>crc_dm_industry</v>
+      </c>
+      <c r="C45" t="str">
+        <v>CRC DM Industry</v>
+      </c>
+      <c r="D45" t="str">
+        <v>BRL</v>
+      </c>
+      <c r="E45" t="b">
+        <v>1</v>
+      </c>
+      <c r="F45">
+        <v>286122.31839448167</v>
+      </c>
+      <c r="G45">
+        <v>241746.33320997993</v>
+      </c>
+      <c r="H45">
+        <v>141551.5847290266</v>
+      </c>
+      <c r="I45">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B46" t="str">
+        <v>crc_dm_downstream</v>
+      </c>
+      <c r="C46" t="str">
+        <v>CRC DM Downstream</v>
+      </c>
+      <c r="D46" t="str">
+        <v>BRL</v>
+      </c>
+      <c r="E46" t="b">
+        <v>1</v>
+      </c>
+      <c r="F46">
+        <v>117390.911</v>
+      </c>
+      <c r="G46">
+        <v>104733.98687029356</v>
+      </c>
+      <c r="H46">
+        <v>67467.37675779735</v>
+      </c>
+      <c r="I46">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B47" t="str">
+        <v>hdg_em_auto</v>
+      </c>
+      <c r="C47" t="str">
+        <v>HDG EM Auto</v>
+      </c>
+      <c r="D47" t="str">
+        <v>BRL</v>
+      </c>
+      <c r="E47" t="b">
+        <v>1</v>
+      </c>
+      <c r="F47">
+        <v>41148.52363473107</v>
+      </c>
+      <c r="G47">
+        <v>43552.244420957155</v>
+      </c>
+      <c r="H47">
+        <v>23560.101535875285</v>
+      </c>
+      <c r="I47">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B48" t="str">
+        <v>hdg_em_industry</v>
+      </c>
+      <c r="C48" t="str">
+        <v>HDG EM Industry</v>
+      </c>
+      <c r="D48" t="str">
+        <v>USD</v>
+      </c>
+      <c r="E48" t="b">
+        <v>0</v>
+      </c>
+      <c r="F48">
+        <v>2599.121</v>
+      </c>
+      <c r="G48">
+        <v>1460.9571992026692</v>
+      </c>
+      <c r="H48">
+        <v>1539.211563265402</v>
+      </c>
+      <c r="I48">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B49" t="str">
+        <v>hdg_dm_auto</v>
+      </c>
+      <c r="C49" t="str">
+        <v>HDG DM Auto</v>
+      </c>
+      <c r="D49" t="str">
+        <v>BRL</v>
+      </c>
+      <c r="E49" t="b">
+        <v>1</v>
+      </c>
+      <c r="F49">
+        <v>463787.28951984947</v>
+      </c>
+      <c r="G49">
+        <v>509632.21143203217</v>
+      </c>
+      <c r="H49">
+        <v>265547.2096431013</v>
+      </c>
+      <c r="I49">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B50" t="str">
+        <v>hdg_dm_industry</v>
+      </c>
+      <c r="C50" t="str">
+        <v>HDG DM Industry</v>
+      </c>
+      <c r="D50" t="str">
+        <v>BRL</v>
+      </c>
+      <c r="E50" t="b">
+        <v>1</v>
+      </c>
+      <c r="F50">
+        <v>438619.17</v>
+      </c>
+      <c r="G50">
+        <v>400262.7377132616</v>
+      </c>
+      <c r="H50">
+        <v>259752.31562280984</v>
+      </c>
+      <c r="I50">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B51" t="str">
+        <v>hdg_dm_downstream</v>
+      </c>
+      <c r="C51" t="str">
+        <v>HDG DM Downstream</v>
+      </c>
+      <c r="D51" t="str">
+        <v>BRL</v>
+      </c>
+      <c r="E51" t="b">
+        <v>1</v>
+      </c>
+      <c r="F51">
+        <v>76159.62108</v>
+      </c>
+      <c r="G51">
+        <v>72400.35218939309</v>
+      </c>
+      <c r="H51">
+        <v>51194.85205203341</v>
+      </c>
+      <c r="I51">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B52" t="str">
+        <v>alzn_dm_industry</v>
+      </c>
+      <c r="C52" t="str">
+        <v>AlZn DM Industry</v>
+      </c>
+      <c r="D52" t="str">
+        <v>BRL</v>
+      </c>
+      <c r="E52" t="b">
+        <v>1</v>
+      </c>
+      <c r="F52">
+        <v>136271.78900000008</v>
+      </c>
+      <c r="G52">
+        <v>140038.4750739659</v>
+      </c>
+      <c r="H52">
+        <v>90465.29575458023</v>
+      </c>
+      <c r="I52">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B53" t="str">
+        <v>alzn_dm_downstream</v>
+      </c>
+      <c r="C53" t="str">
+        <v>ALZn DM Downstream</v>
+      </c>
+      <c r="D53" t="str">
+        <v>BRL</v>
+      </c>
+      <c r="E53" t="b">
+        <v>1</v>
+      </c>
+      <c r="F53">
+        <v>88523.36700000001</v>
+      </c>
+      <c r="G53">
+        <v>104845.59585986432</v>
+      </c>
+      <c r="H53">
+        <v>65848.93065429507</v>
+      </c>
+      <c r="I53">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B54" t="str">
+        <v>usibor_dm_auto</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Usibor DM Auto</v>
+      </c>
+      <c r="D54" t="str">
+        <v>BRL</v>
+      </c>
+      <c r="E54" t="b">
+        <v>1</v>
+      </c>
+      <c r="F54">
+        <v>99323.02080009198</v>
+      </c>
+      <c r="G54">
+        <v>137190.0543820729</v>
+      </c>
+      <c r="H54">
+        <v>56896.46654510919</v>
+      </c>
+      <c r="I54">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B55" t="str">
+        <v>alsi_dm_industry</v>
+      </c>
+      <c r="C55" t="str">
+        <v>AlSi DM Industry</v>
+      </c>
+      <c r="D55" t="str">
+        <v>BRL</v>
+      </c>
+      <c r="E55" t="b">
+        <v>1</v>
+      </c>
+      <c r="F55">
+        <v>7661.225</v>
+      </c>
+      <c r="G55">
+        <v>6281.118265921143</v>
+      </c>
+      <c r="H55">
+        <v>4388.676747804378</v>
+      </c>
+      <c r="I55">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B56" t="str">
+        <v>auto_imports_pp_dm</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Auto Imports/PP DM</v>
+      </c>
+      <c r="D56" t="str">
+        <v>BRL</v>
+      </c>
+      <c r="E56" t="b">
+        <v>1</v>
+      </c>
+      <c r="F56">
+        <v>3627.2928948158055</v>
+      </c>
+      <c r="G56">
+        <v>7076.0467377956575</v>
+      </c>
+      <c r="H56">
+        <v>2408.012156632061</v>
+      </c>
+      <c r="I56">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B57" t="str">
+        <v>magnelis_dm_industry</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Magnelis DM Industry</v>
+      </c>
+      <c r="D57" t="str">
+        <v>USD</v>
+      </c>
+      <c r="E57" t="b">
+        <v>0</v>
+      </c>
+      <c r="F57">
+        <v>10000</v>
+      </c>
+      <c r="G57">
+        <v>4812.364106791682</v>
+      </c>
+      <c r="H57">
+        <v>6638.593095345668</v>
+      </c>
+      <c r="I57">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B58" t="str">
+        <v>industry_imports</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Industry Imports</v>
+      </c>
+      <c r="D58" t="str">
+        <v>BRL</v>
+      </c>
+      <c r="E58" t="b">
+        <v>1</v>
+      </c>
+      <c r="F58">
+        <v>17169.268000000007</v>
+      </c>
+      <c r="G58">
+        <v>17289.10920878557</v>
+      </c>
+      <c r="H58">
+        <v>11397.978399693939</v>
+      </c>
+      <c r="I58">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B59" t="str">
+        <v>magnelis_dm_downstream</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Magnelis DM Downstream</v>
+      </c>
+      <c r="D59" t="str">
+        <v>BRL</v>
+      </c>
+      <c r="E59" t="b">
+        <v>1</v>
+      </c>
+      <c r="F59">
+        <v>7002.88</v>
+      </c>
+      <c r="G59">
+        <v>7055.529422195022</v>
+      </c>
+      <c r="H59">
+        <v>4648.927081553427</v>
+      </c>
+      <c r="I59">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I59"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:E19"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>chave</v>
+        <v>cenario_id</v>
       </c>
       <c r="B1" t="str">
-        <v>descricao</v>
+        <v>categoria</v>
+      </c>
+      <c r="C1" t="str">
+        <v>montante_kusd</v>
+      </c>
+      <c r="D1" t="str">
+        <v>usd</v>
+      </c>
+      <c r="E1" t="str">
+        <v>ordem</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ebitda</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B2" t="str">
-        <v>EBITDA do cenário (MUSD)</v>
+        <v>Labor</v>
+      </c>
+      <c r="C2">
+        <v>290502.46044270345</v>
+      </c>
+      <c r="D2" t="b">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>vol_mix</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B3" t="str">
-        <v>Volume &amp; Mix — nível acumulado vs referência (MUSD)</v>
+        <v>R&amp;M</v>
+      </c>
+      <c r="C3">
+        <v>162910.3754855557</v>
+      </c>
+      <c r="D3" t="b">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>selling_price</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B4" t="str">
-        <v>Preço de venda — nível acumulado vs referência (MUSD)</v>
+        <v>R&amp;M USD</v>
+      </c>
+      <c r="C4">
+        <v>455.3196888888888</v>
+      </c>
+      <c r="D4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>input_price</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B5" t="str">
-        <v>Preço de insumos — nível acumulado vs referência (MUSD)</v>
+        <v>SG&amp;A</v>
+      </c>
+      <c r="C5">
+        <v>36445.369559722225</v>
+      </c>
+      <c r="D5" t="b">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>usage</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B6" t="str">
-        <v>Consumo (Usage) — nível acumulado vs referência (MUSD)</v>
+        <v>SG&amp;A USD</v>
+      </c>
+      <c r="C6">
+        <v>4329.657142592592</v>
+      </c>
+      <c r="D6" t="b">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>fixed_cost</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B7" t="str">
-        <v>Custo fixo — nível acumulado vs referência (MUSD)</v>
+        <v>SG&amp;A NC</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7" t="b">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>forex</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B8" t="str">
-        <v>Câmbio — nível acumulado vs referência (MUSD)</v>
+        <v>SG&amp;A NC USD</v>
+      </c>
+      <c r="C8">
+        <v>3800.225814814815</v>
+      </c>
+      <c r="D8" t="b">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>sv_others</v>
+        <v>fy26_fy_budget</v>
       </c>
       <c r="B9" t="str">
-        <v>Estoque / Outros — nível acumulado vs referência (MUSD)</v>
+        <v>Production</v>
+      </c>
+      <c r="C9">
+        <v>133766.8745303331</v>
+      </c>
+      <c r="D9" t="b">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>fy26_fy_budget</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Production USD</v>
+      </c>
+      <c r="C10">
+        <v>57260.893387037046</v>
+      </c>
+      <c r="D10" t="b">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Labor</v>
+      </c>
+      <c r="C11">
+        <v>335945.75819845067</v>
+      </c>
+      <c r="D11" t="b">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B12" t="str">
+        <v>R&amp;M</v>
+      </c>
+      <c r="C12">
+        <v>173542.33833959477</v>
+      </c>
+      <c r="D12" t="b">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B13" t="str">
+        <v>R&amp;M USD</v>
+      </c>
+      <c r="C13">
+        <v>476.59812750037713</v>
+      </c>
+      <c r="D13" t="b">
+        <v>1</v>
+      </c>
+      <c r="E13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B14" t="str">
+        <v>SG&amp;A</v>
+      </c>
+      <c r="C14">
+        <v>39799.933372505184</v>
+      </c>
+      <c r="D14" t="b">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B15" t="str">
+        <v>SG&amp;A USD</v>
+      </c>
+      <c r="C15">
+        <v>4366.799716101096</v>
+      </c>
+      <c r="D15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E15">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B16" t="str">
+        <v>SG&amp;A NC</v>
+      </c>
+      <c r="C16">
+        <v>0</v>
+      </c>
+      <c r="D16" t="b">
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B17" t="str">
+        <v>SG&amp;A NC USD</v>
+      </c>
+      <c r="C17">
+        <v>4339.968285153967</v>
+      </c>
+      <c r="D17" t="b">
+        <v>1</v>
+      </c>
+      <c r="E17">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Production</v>
+      </c>
+      <c r="C18">
+        <v>137770.91554820424</v>
+      </c>
+      <c r="D18" t="b">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Production USD</v>
+      </c>
+      <c r="C19">
+        <v>56306.50454336941</v>
+      </c>
+      <c r="D19" t="b">
+        <v>1</v>
+      </c>
+      <c r="E19">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E19"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F33"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>cenario_id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>item</v>
+      </c>
+      <c r="C1" t="str">
+        <v>preco_usd</v>
+      </c>
+      <c r="D1" t="str">
+        <v>rendimento</v>
+      </c>
+      <c r="E1" t="str">
+        <v>montante_kusd</v>
+      </c>
+      <c r="F1" t="str">
+        <v>ordem</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>fy26_fy_budget</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Coal</v>
+      </c>
+      <c r="C2">
+        <v>192.44907581258093</v>
+      </c>
+      <c r="D2">
+        <v>0.39731562421943</v>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>fy26_fy_budget</v>
+      </c>
+      <c r="B3" t="str">
+        <v>PCI</v>
+      </c>
+      <c r="C3">
+        <v>193.479079981596</v>
+      </c>
+      <c r="D3">
+        <v>0.27102848197245</v>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>fy26_fy_budget</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Others (Antracito)</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>fy26_fy_budget</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Purchased coke</v>
+      </c>
+      <c r="C5">
+        <v>312.929445101365</v>
+      </c>
+      <c r="D5">
+        <v>0.01407606697906</v>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>fy26_fy_budget</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Fines</v>
+      </c>
+      <c r="C6">
+        <v>72.7248055631426</v>
+      </c>
+      <c r="D6">
+        <v>0.50546147907213</v>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>fy26_fy_budget</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Pellets</v>
+      </c>
+      <c r="C7">
+        <v>121.43893018053701</v>
+      </c>
+      <c r="D7">
+        <v>0.78699859872351</v>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>fy26_fy_budget</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Lumps</v>
+      </c>
+      <c r="C8">
+        <v>82.1839244705543</v>
+      </c>
+      <c r="D8">
+        <v>0.2207053984765</v>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>fy26_fy_budget</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Alloys</v>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>fy26_fy_budget</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Zinc</v>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>fy26_fy_budget</v>
+      </c>
+      <c r="B11" t="str">
+        <v>AMS allocation fee</v>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>fy26_fy_budget</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Natural Gas</v>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>fy26_fy_budget</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Fluxes</v>
+      </c>
+      <c r="C13" t="str">
+        <v/>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>fy26_fy_budget</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Energy</v>
+      </c>
+      <c r="C14" t="str">
+        <v/>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>fy26_fy_budget</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Refractories</v>
+      </c>
+      <c r="C15" t="str">
+        <v/>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>fy26_fy_budget</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Var. contractors</v>
+      </c>
+      <c r="C16" t="str">
+        <v/>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>fy26_fy_budget</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Freight rate</v>
+      </c>
+      <c r="C17" t="str">
+        <v/>
+      </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
+      <c r="E17">
+        <v>0</v>
+      </c>
+      <c r="F17">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Coal</v>
+      </c>
+      <c r="C18">
+        <v>209.83033201184605</v>
+      </c>
+      <c r="D18">
+        <v>0.39731562421943</v>
+      </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B19" t="str">
+        <v>PCI</v>
+      </c>
+      <c r="C19">
+        <v>218.48672314443104</v>
+      </c>
+      <c r="D19">
+        <v>0.27102848197245</v>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+      <c r="F19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Others (Antracito)</v>
+      </c>
+      <c r="C20">
+        <v>0</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Purchased coke</v>
+      </c>
+      <c r="C21">
+        <v>340.6182272150431</v>
+      </c>
+      <c r="D21">
+        <v>0.01407606697906</v>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+      <c r="F21">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Fines</v>
+      </c>
+      <c r="C22">
+        <v>75.8038935935645</v>
+      </c>
+      <c r="D22">
+        <v>0.50546147907213</v>
+      </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
+      <c r="F22">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Pellets</v>
+      </c>
+      <c r="C23">
+        <v>128.957925964685</v>
+      </c>
+      <c r="D23">
+        <v>0.78699859872351</v>
+      </c>
+      <c r="E23" t="str">
+        <v/>
+      </c>
+      <c r="F23">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Lumps</v>
+      </c>
+      <c r="C24">
+        <v>83.4702474919854</v>
+      </c>
+      <c r="D24">
+        <v>0.2207053984765</v>
+      </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
+      <c r="F24">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Alloys</v>
+      </c>
+      <c r="C25" t="str">
+        <v/>
+      </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
+      <c r="E25">
+        <v>-12014.33914384416</v>
+      </c>
+      <c r="F25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Zinc</v>
+      </c>
+      <c r="C26" t="str">
+        <v/>
+      </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
+      <c r="E26">
+        <v>-11030</v>
+      </c>
+      <c r="F26">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B27" t="str">
+        <v>AMS allocation fee</v>
+      </c>
+      <c r="C27" t="str">
+        <v/>
+      </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
+      <c r="E27">
+        <v>6564.3217252063005</v>
+      </c>
+      <c r="F27">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Natural Gas</v>
+      </c>
+      <c r="C28" t="str">
+        <v/>
+      </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
+      <c r="E28">
+        <v>206.90204446817884</v>
+      </c>
+      <c r="F28">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Fluxes</v>
+      </c>
+      <c r="C29" t="str">
+        <v/>
+      </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
+      <c r="E29">
+        <v>-7030</v>
+      </c>
+      <c r="F29">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Energy</v>
+      </c>
+      <c r="C30" t="str">
+        <v/>
+      </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
+      <c r="E30">
+        <v>-2000</v>
+      </c>
+      <c r="F30">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Refractories</v>
+      </c>
+      <c r="C31" t="str">
+        <v/>
+      </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
+      <c r="E31">
+        <v>0</v>
+      </c>
+      <c r="F31">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Var. contractors</v>
+      </c>
+      <c r="C32" t="str">
+        <v/>
+      </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
+      <c r="E32">
+        <v>0</v>
+      </c>
+      <c r="F32">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Freight rate</v>
+      </c>
+      <c r="C33" t="str">
+        <v/>
+      </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
+      <c r="E33">
+        <v>0</v>
+      </c>
+      <c r="F33">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F33"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>cenario_id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>alavanca</v>
+      </c>
+      <c r="C1" t="str">
+        <v>linha</v>
+      </c>
+      <c r="D1" t="str">
+        <v>montante_kusd</v>
+      </c>
+      <c r="E1" t="str">
+        <v>ordem</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>fy26_fy_budget</v>
+      </c>
+      <c r="B2" t="str">
+        <v>usage</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Consumo de insumos</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>fy26_fy_budget</v>
+      </c>
+      <c r="B3" t="str">
+        <v>others</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Logistic / VAT</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>fy26_fy_budget</v>
+      </c>
+      <c r="B4" t="str">
+        <v>stock_variation</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Non Steel</v>
+      </c>
+      <c r="D4">
+        <v>12000</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>fy26_fy_budget</v>
+      </c>
+      <c r="B5" t="str">
+        <v>stock_variation</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Legal contingency</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>fy26_fy_budget</v>
+      </c>
+      <c r="B6" t="str">
+        <v>stock_variation</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Slowmoving</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>fy26_fy_budget</v>
+      </c>
+      <c r="B7" t="str">
+        <v>stock_variation</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Invest-ES</v>
+      </c>
+      <c r="D7">
+        <v>134784.708518517</v>
+      </c>
+      <c r="E7">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>fy26_fy_budget</v>
+      </c>
+      <c r="B8" t="str">
+        <v>stock_variation</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Ajuste QM (reclamação cliente)</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B9" t="str">
+        <v>usage</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Consumo de insumos</v>
+      </c>
+      <c r="D9">
+        <v>-12829.343372386798</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B10" t="str">
+        <v>others</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Logistic / VAT</v>
+      </c>
+      <c r="D10">
+        <v>-5764.020362938623</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B11" t="str">
+        <v>stock_variation</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Non Steel</v>
+      </c>
+      <c r="D11">
+        <v>18490.46697130281</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B12" t="str">
+        <v>stock_variation</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Legal contingency</v>
+      </c>
+      <c r="D12">
+        <v>149.79323466958516</v>
+      </c>
+      <c r="E12">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B13" t="str">
+        <v>stock_variation</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Slowmoving</v>
+      </c>
+      <c r="D13">
+        <v>-2604.118710140672</v>
+      </c>
+      <c r="E13">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B14" t="str">
+        <v>stock_variation</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Invest-ES</v>
+      </c>
+      <c r="D14">
+        <v>129888.14456308608</v>
+      </c>
+      <c r="E14">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>fy26_fy_mrf7</v>
+      </c>
+      <c r="B15" t="str">
+        <v>stock_variation</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Ajuste QM (reclamação cliente)</v>
+      </c>
+      <c r="D15">
+        <v>-3000</v>
+      </c>
+      <c r="E15">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>